<commit_message>
testes: registro com SEQ coletado após as sessões
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcvsyGAzxjz3qNYZ87Tbjb
</commit_message>
<xml_diff>
--- a/testes/registro-testes.xlsx
+++ b/testes/registro-testes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felipelatinisoffiatti/Documents/Felipe/02. Pessoal/02. Estudo/02. Inteli/03. Artigos &amp; Documentos/02. Documentos Módulos/Módulo. 03/Case Instituto Ebenezer/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nelsonsouzaneto/Library/Mobile Documents/com~apple~CloudDocs/ACADEMIA/INTELI/MBA 2026/MODULO 3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1405B99-6AC2-A748-BE82-2FA3338D83CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B2125E7-6116-F84A-8CBB-F659D8C65FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29240" windowHeight="16980" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29240" windowHeight="16980" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instruções" sheetId="1" r:id="rId1"/>
@@ -562,25 +562,25 @@
       <sz val="14"/>
       <color rgb="FF006255"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -674,10 +674,10 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1121,10 +1121,10 @@
       <c r="D2" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="14" t="s">
         <v>151</v>
       </c>
       <c r="G2" s="8" t="s">
@@ -1148,10 +1148,10 @@
       <c r="D3" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="14" t="s">
         <v>159</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -1175,10 +1175,10 @@
       <c r="D4" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="14" t="s">
         <v>160</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -1274,7 +1274,9 @@
       <c r="G2" s="8">
         <v>57</v>
       </c>
-      <c r="H2" s="8"/>
+      <c r="H2" s="8">
+        <v>6</v>
+      </c>
       <c r="I2" s="8"/>
       <c r="J2" s="8"/>
     </row>
@@ -1300,9 +1302,11 @@
       <c r="G3" s="8">
         <v>212</v>
       </c>
-      <c r="H3" s="8"/>
+      <c r="H3" s="8">
+        <v>3</v>
+      </c>
       <c r="I3" s="8"/>
-      <c r="J3" s="15" t="s">
+      <c r="J3" s="14" t="s">
         <v>156</v>
       </c>
     </row>
@@ -1328,7 +1332,9 @@
       <c r="G4" s="8">
         <v>12</v>
       </c>
-      <c r="H4" s="8"/>
+      <c r="H4" s="8">
+        <v>7</v>
+      </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
     </row>
@@ -1354,7 +1360,9 @@
       <c r="G5" s="8">
         <v>183</v>
       </c>
-      <c r="H5" s="8"/>
+      <c r="H5" s="8">
+        <v>6</v>
+      </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
     </row>
@@ -1380,7 +1388,9 @@
       <c r="G6" s="8">
         <v>62</v>
       </c>
-      <c r="H6" s="8"/>
+      <c r="H6" s="8">
+        <v>5</v>
+      </c>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
     </row>
@@ -1406,7 +1416,9 @@
       <c r="G7" s="8">
         <v>7</v>
       </c>
-      <c r="H7" s="8"/>
+      <c r="H7" s="8">
+        <v>7</v>
+      </c>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
     </row>
@@ -1432,7 +1444,9 @@
       <c r="G8" s="8">
         <v>22</v>
       </c>
-      <c r="H8" s="8"/>
+      <c r="H8" s="8">
+        <v>5</v>
+      </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
     </row>
@@ -1458,7 +1472,9 @@
       <c r="G9" s="8">
         <v>18</v>
       </c>
-      <c r="H9" s="8"/>
+      <c r="H9" s="8">
+        <v>5</v>
+      </c>
       <c r="I9" s="8"/>
       <c r="J9" s="8"/>
     </row>
@@ -1481,10 +1497,12 @@
       <c r="F10" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="G10" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="H10" s="8"/>
+      <c r="H10" s="8">
+        <v>2</v>
+      </c>
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
     </row>
@@ -1510,7 +1528,9 @@
       <c r="G11" s="8">
         <v>21</v>
       </c>
-      <c r="H11" s="8"/>
+      <c r="H11" s="8">
+        <v>5</v>
+      </c>
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
     </row>
@@ -1536,7 +1556,9 @@
       <c r="G12" s="8">
         <v>11</v>
       </c>
-      <c r="H12" s="8"/>
+      <c r="H12" s="8">
+        <v>4</v>
+      </c>
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
@@ -1562,7 +1584,9 @@
       <c r="G13" s="8">
         <v>14</v>
       </c>
-      <c r="H13" s="8"/>
+      <c r="H13" s="8">
+        <v>5</v>
+      </c>
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
@@ -1879,13 +1903,13 @@
       <c r="A2" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="14" t="s">
         <v>21</v>
       </c>
       <c r="E2" s="8">
@@ -1894,13 +1918,13 @@
       <c r="F2" s="8">
         <v>3</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="14" t="s">
         <v>163</v>
       </c>
       <c r="H2" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="14" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2268,16 +2292,16 @@
       <c r="A7" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="B7" s="13" t="str">
+      <c r="B7" s="13">
         <f>IF(COUNT(Tarefas!$H$2:$H$13)=0,"",AVERAGE(Tarefas!$H$2:$H$13))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="C7" s="13">
         <v>5.5</v>
       </c>
       <c r="D7" s="1" t="str">
         <f>IF(B7="","Aguardando",IF(B7&gt;=C7,"Atende","Não atende"))</f>
-        <v>Aguardando</v>
+        <v>Não atende</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>135</v>
@@ -2376,9 +2400,9 @@
         <f>IF(COUNTIFS(Tarefas!$B$2:$B$13,"P1",Tarefas!$F$2:$F$13,"&lt;&gt;")=0,"",COUNTIFS(Tarefas!$B$2:$B$13,"P1",Tarefas!$F$2:$F$13,"S")/COUNTIFS(Tarefas!$B$2:$B$13,"P1",Tarefas!$F$2:$F$13,"&lt;&gt;"))</f>
         <v>0.75</v>
       </c>
-      <c r="C14" s="13" t="str">
+      <c r="C14" s="13">
         <f>IF(COUNTIFS(Tarefas!$B$2:$B$13,"P1",Tarefas!$H$2:$H$13,"&lt;&gt;")=0,"",AVERAGEIFS(Tarefas!$H$2:$H$13,Tarefas!$B$2:$B$13,"P1"))</f>
-        <v/>
+        <v>5.5</v>
       </c>
       <c r="D14" s="13">
         <f>SUS!C12</f>
@@ -2394,9 +2418,9 @@
         <f>IF(COUNTIFS(Tarefas!$B$2:$B$13,"P2",Tarefas!$F$2:$F$13,"&lt;&gt;")=0,"",COUNTIFS(Tarefas!$B$2:$B$13,"P2",Tarefas!$F$2:$F$13,"S")/COUNTIFS(Tarefas!$B$2:$B$13,"P2",Tarefas!$F$2:$F$13,"&lt;&gt;"))</f>
         <v>0.5</v>
       </c>
-      <c r="C15" s="13" t="str">
+      <c r="C15" s="13">
         <f>IF(COUNTIFS(Tarefas!$B$2:$B$13,"P2",Tarefas!$H$2:$H$13,"&lt;&gt;")=0,"",AVERAGEIFS(Tarefas!$H$2:$H$13,Tarefas!$B$2:$B$13,"P2"))</f>
-        <v/>
+        <v>5.5</v>
       </c>
       <c r="D15" s="13">
         <f>SUS!D12</f>
@@ -2412,9 +2436,9 @@
         <f>IF(COUNTIFS(Tarefas!$B$2:$B$13,"P3",Tarefas!$F$2:$F$13,"&lt;&gt;")=0,"",COUNTIFS(Tarefas!$B$2:$B$13,"P3",Tarefas!$F$2:$F$13,"S")/COUNTIFS(Tarefas!$B$2:$B$13,"P3",Tarefas!$F$2:$F$13,"&lt;&gt;"))</f>
         <v>0.75</v>
       </c>
-      <c r="C16" s="13" t="str">
+      <c r="C16" s="13">
         <f>IF(COUNTIFS(Tarefas!$B$2:$B$13,"P3",Tarefas!$H$2:$H$13,"&lt;&gt;")=0,"",AVERAGEIFS(Tarefas!$H$2:$H$13,Tarefas!$B$2:$B$13,"P3"))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="D16" s="13">
         <f>SUS!E12</f>
@@ -2423,13 +2447,13 @@
       <c r="E16" s="1"/>
     </row>
     <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>